<commit_message>
Fix sheet name and group number type for Yandex Direct import
</commit_message>
<xml_diff>
--- a/direct_voronezh_krovstroyrf.xlsx
+++ b/direct_voronezh_krovstroyrf.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Кампания" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -596,10 +596,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B3" t="n">
+        <v>1</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -719,10 +717,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B4" t="n">
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -842,10 +838,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B5" t="n">
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -965,10 +959,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B6" t="n">
+        <v>1</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -1088,10 +1080,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B7" t="n">
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -1211,10 +1201,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B8" t="n">
+        <v>1</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1334,10 +1322,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B9" t="n">
+        <v>1</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1457,10 +1443,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B10" t="n">
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1580,10 +1564,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B11" t="n">
+        <v>1</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1703,10 +1685,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B12" t="n">
+        <v>1</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1826,10 +1806,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B13" t="n">
+        <v>1</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1873,10 +1851,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B14" t="n">
+        <v>1</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -1920,10 +1896,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B15" t="n">
+        <v>1</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1967,10 +1941,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B16" t="n">
+        <v>1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -2014,10 +1986,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B17" t="n">
+        <v>1</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -2061,10 +2031,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B18" t="n">
+        <v>1</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -2108,10 +2076,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B19" t="n">
+        <v>1</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2155,10 +2121,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B20" t="n">
+        <v>1</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2202,10 +2166,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B21" t="n">
+        <v>1</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2249,10 +2211,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B22" t="n">
+        <v>1</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2296,10 +2256,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B23" t="n">
+        <v>1</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2343,10 +2301,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B24" t="n">
+        <v>1</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -2390,10 +2346,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B25" t="n">
+        <v>1</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2437,10 +2391,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B26" t="n">
+        <v>1</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2484,10 +2436,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B27" t="n">
+        <v>1</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2531,10 +2481,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B28" t="n">
+        <v>1</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2578,10 +2526,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B29" t="n">
+        <v>1</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2625,10 +2571,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B30" t="n">
+        <v>1</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -2672,10 +2616,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B31" t="n">
+        <v>1</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -2719,10 +2661,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B32" t="n">
+        <v>1</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -2766,10 +2706,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B33" t="n">
+        <v>1</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -2813,10 +2751,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B34" t="n">
+        <v>1</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -2860,10 +2796,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B35" t="n">
+        <v>1</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -2907,10 +2841,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B36" t="n">
+        <v>1</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -2954,10 +2886,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B37" t="n">
+        <v>1</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3001,10 +2931,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B38" t="n">
+        <v>1</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3048,10 +2976,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B39" t="n">
+        <v>1</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3095,10 +3021,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B40" t="n">
+        <v>1</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -3142,10 +3066,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B41" t="n">
+        <v>1</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -3189,10 +3111,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B42" t="n">
+        <v>1</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -3236,10 +3156,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B43" t="n">
+        <v>1</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -3283,10 +3201,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B44" t="n">
+        <v>1</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -3330,10 +3246,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B45" t="n">
+        <v>1</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -3377,10 +3291,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B46" t="n">
+        <v>1</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -3424,10 +3336,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B47" t="n">
+        <v>1</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -3471,10 +3381,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B48" t="n">
+        <v>1</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -3518,10 +3426,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B49" t="n">
+        <v>1</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -3565,10 +3471,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B50" t="n">
+        <v>1</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -3612,10 +3516,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B51" t="n">
+        <v>1</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -3659,10 +3561,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B52" t="n">
+        <v>1</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -3706,10 +3606,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B53" t="n">
+        <v>1</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -3753,10 +3651,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B54" t="n">
+        <v>1</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -3800,10 +3696,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B55" t="n">
+        <v>1</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -3847,10 +3741,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B56" t="n">
+        <v>1</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -3894,10 +3786,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B57" t="n">
+        <v>1</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -3941,10 +3831,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B58" t="n">
+        <v>1</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -3988,10 +3876,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B59" t="n">
+        <v>1</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -4035,10 +3921,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B60" t="n">
+        <v>1</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -4082,10 +3966,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B61" t="n">
+        <v>1</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -4129,10 +4011,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B62" t="n">
+        <v>1</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -4176,10 +4056,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B63" t="n">
+        <v>1</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -4223,10 +4101,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B64" t="n">
+        <v>1</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -4270,10 +4146,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B65" t="n">
+        <v>1</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -4317,10 +4191,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B66" t="n">
+        <v>1</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -4364,10 +4236,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B67" t="n">
+        <v>1</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -4411,10 +4281,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B68" t="n">
+        <v>1</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -4458,10 +4326,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B69" t="n">
+        <v>1</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -4505,10 +4371,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B70" t="n">
+        <v>1</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -4552,10 +4416,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B71" t="n">
+        <v>1</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -4599,10 +4461,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B72" t="n">
+        <v>1</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -4646,10 +4506,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B73" t="n">
+        <v>1</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -4693,10 +4551,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B74" t="n">
+        <v>1</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -4740,10 +4596,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B75" t="n">
+        <v>1</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -4787,10 +4641,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B76" t="n">
+        <v>1</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -4834,10 +4686,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B77" t="n">
+        <v>1</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -4881,10 +4731,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B78" t="n">
+        <v>1</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -4928,10 +4776,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B79" t="n">
+        <v>1</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -4975,10 +4821,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B80" t="n">
+        <v>1</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -5022,10 +4866,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B81" t="n">
+        <v>1</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -5069,10 +4911,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B82" t="n">
+        <v>1</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -5116,10 +4956,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B83" t="n">
+        <v>1</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -5163,10 +5001,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B84" t="n">
+        <v>1</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -5210,10 +5046,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B85" t="n">
+        <v>1</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -5257,10 +5091,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B86" t="n">
+        <v>1</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -5304,10 +5136,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B87" t="n">
+        <v>1</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -5351,10 +5181,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B88" t="n">
+        <v>1</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -5398,10 +5226,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B89" t="n">
+        <v>1</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -5445,10 +5271,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B90" t="n">
+        <v>1</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -5492,10 +5316,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B91" t="n">
+        <v>1</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -5539,10 +5361,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="B92" t="n">
+        <v>1</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -5586,10 +5406,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B93" t="n">
+        <v>2</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -5709,10 +5527,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B94" t="n">
+        <v>2</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -5832,10 +5648,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B95" t="n">
+        <v>2</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -5955,10 +5769,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B96" t="n">
+        <v>2</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -6078,10 +5890,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B97" t="n">
+        <v>2</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -6201,10 +6011,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B98" t="n">
+        <v>2</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -6324,10 +6132,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B99" t="n">
+        <v>2</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -6447,10 +6253,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B100" t="n">
+        <v>2</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -6570,10 +6374,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B101" t="n">
+        <v>2</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -6693,10 +6495,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B102" t="n">
+        <v>2</v>
       </c>
       <c r="C102" t="inlineStr">
         <is>
@@ -6816,10 +6616,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B103" t="n">
+        <v>2</v>
       </c>
       <c r="C103" t="inlineStr">
         <is>
@@ -6863,10 +6661,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B104" t="n">
+        <v>2</v>
       </c>
       <c r="C104" t="inlineStr">
         <is>
@@ -6910,10 +6706,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B105" t="n">
+        <v>2</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -6957,10 +6751,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B106" t="n">
+        <v>2</v>
       </c>
       <c r="C106" t="inlineStr">
         <is>
@@ -7004,10 +6796,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B107" t="n">
+        <v>2</v>
       </c>
       <c r="C107" t="inlineStr">
         <is>
@@ -7051,10 +6841,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B108" t="n">
+        <v>2</v>
       </c>
       <c r="C108" t="inlineStr">
         <is>
@@ -7098,10 +6886,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B109" t="n">
+        <v>2</v>
       </c>
       <c r="C109" t="inlineStr">
         <is>
@@ -7145,10 +6931,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B110" t="n">
+        <v>2</v>
       </c>
       <c r="C110" t="inlineStr">
         <is>
@@ -7192,10 +6976,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B111" t="n">
+        <v>2</v>
       </c>
       <c r="C111" t="inlineStr">
         <is>
@@ -7239,10 +7021,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B112" t="n">
+        <v>2</v>
       </c>
       <c r="C112" t="inlineStr">
         <is>
@@ -7286,10 +7066,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B113" t="n">
+        <v>2</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -7333,10 +7111,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B114" t="n">
+        <v>2</v>
       </c>
       <c r="C114" t="inlineStr">
         <is>
@@ -7380,10 +7156,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B115" t="n">
+        <v>2</v>
       </c>
       <c r="C115" t="inlineStr">
         <is>
@@ -7427,10 +7201,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B116" t="n">
+        <v>2</v>
       </c>
       <c r="C116" t="inlineStr">
         <is>
@@ -7474,10 +7246,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B117" t="n">
+        <v>2</v>
       </c>
       <c r="C117" t="inlineStr">
         <is>
@@ -7521,10 +7291,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B118" t="n">
+        <v>2</v>
       </c>
       <c r="C118" t="inlineStr">
         <is>
@@ -7568,10 +7336,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B119" t="n">
+        <v>2</v>
       </c>
       <c r="C119" t="inlineStr">
         <is>
@@ -7615,10 +7381,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B120" t="n">
+        <v>2</v>
       </c>
       <c r="C120" t="inlineStr">
         <is>
@@ -7662,10 +7426,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B121" t="n">
+        <v>2</v>
       </c>
       <c r="C121" t="inlineStr">
         <is>
@@ -7709,10 +7471,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B122" t="n">
+        <v>2</v>
       </c>
       <c r="C122" t="inlineStr">
         <is>
@@ -7756,10 +7516,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B123" t="n">
+        <v>2</v>
       </c>
       <c r="C123" t="inlineStr">
         <is>
@@ -7803,10 +7561,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B124" t="n">
+        <v>2</v>
       </c>
       <c r="C124" t="inlineStr">
         <is>
@@ -7850,10 +7606,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B125" t="n">
+        <v>2</v>
       </c>
       <c r="C125" t="inlineStr">
         <is>
@@ -7897,10 +7651,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B126" t="n">
+        <v>2</v>
       </c>
       <c r="C126" t="inlineStr">
         <is>
@@ -7944,10 +7696,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B127" t="n">
+        <v>2</v>
       </c>
       <c r="C127" t="inlineStr">
         <is>
@@ -7991,10 +7741,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B128" t="n">
+        <v>2</v>
       </c>
       <c r="C128" t="inlineStr">
         <is>
@@ -8038,10 +7786,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B129" t="n">
+        <v>2</v>
       </c>
       <c r="C129" t="inlineStr">
         <is>
@@ -8085,10 +7831,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B130" t="n">
+        <v>2</v>
       </c>
       <c r="C130" t="inlineStr">
         <is>
@@ -8132,10 +7876,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B131" t="n">
+        <v>2</v>
       </c>
       <c r="C131" t="inlineStr">
         <is>
@@ -8179,10 +7921,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B132" t="n">
+        <v>2</v>
       </c>
       <c r="C132" t="inlineStr">
         <is>
@@ -8226,10 +7966,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B133" t="n">
+        <v>2</v>
       </c>
       <c r="C133" t="inlineStr">
         <is>
@@ -8273,10 +8011,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B134" t="n">
+        <v>2</v>
       </c>
       <c r="C134" t="inlineStr">
         <is>
@@ -8320,10 +8056,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B135" t="n">
+        <v>2</v>
       </c>
       <c r="C135" t="inlineStr">
         <is>
@@ -8367,10 +8101,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B136" t="n">
+        <v>2</v>
       </c>
       <c r="C136" t="inlineStr">
         <is>
@@ -8414,10 +8146,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B137" t="n">
+        <v>2</v>
       </c>
       <c r="C137" t="inlineStr">
         <is>
@@ -8461,10 +8191,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B138" t="n">
+        <v>2</v>
       </c>
       <c r="C138" t="inlineStr">
         <is>
@@ -8508,10 +8236,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B139" t="n">
+        <v>2</v>
       </c>
       <c r="C139" t="inlineStr">
         <is>
@@ -8555,10 +8281,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B140" t="n">
+        <v>2</v>
       </c>
       <c r="C140" t="inlineStr">
         <is>
@@ -8602,10 +8326,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B141" t="n">
+        <v>2</v>
       </c>
       <c r="C141" t="inlineStr">
         <is>
@@ -8649,10 +8371,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B142" t="n">
+        <v>2</v>
       </c>
       <c r="C142" t="inlineStr">
         <is>
@@ -8696,10 +8416,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B143" t="n">
+        <v>2</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
@@ -8743,10 +8461,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B144" t="n">
+        <v>2</v>
       </c>
       <c r="C144" t="inlineStr">
         <is>
@@ -8790,10 +8506,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B145" t="n">
+        <v>2</v>
       </c>
       <c r="C145" t="inlineStr">
         <is>
@@ -8837,10 +8551,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B146" t="n">
+        <v>2</v>
       </c>
       <c r="C146" t="inlineStr">
         <is>
@@ -8884,10 +8596,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B147" t="n">
+        <v>2</v>
       </c>
       <c r="C147" t="inlineStr">
         <is>
@@ -8931,10 +8641,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B148" t="n">
+        <v>2</v>
       </c>
       <c r="C148" t="inlineStr">
         <is>
@@ -8978,10 +8686,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B149" t="n">
+        <v>2</v>
       </c>
       <c r="C149" t="inlineStr">
         <is>
@@ -9025,10 +8731,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B150" t="n">
+        <v>2</v>
       </c>
       <c r="C150" t="inlineStr">
         <is>
@@ -9072,10 +8776,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B151" t="n">
+        <v>2</v>
       </c>
       <c r="C151" t="inlineStr">
         <is>
@@ -9119,10 +8821,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B152" t="n">
+        <v>2</v>
       </c>
       <c r="C152" t="inlineStr">
         <is>
@@ -9166,10 +8866,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B153" t="n">
+        <v>2</v>
       </c>
       <c r="C153" t="inlineStr">
         <is>
@@ -9213,10 +8911,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B154" t="n">
+        <v>2</v>
       </c>
       <c r="C154" t="inlineStr">
         <is>
@@ -9260,10 +8956,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B155" t="n">
+        <v>2</v>
       </c>
       <c r="C155" t="inlineStr">
         <is>
@@ -9307,10 +9001,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B156" t="n">
+        <v>2</v>
       </c>
       <c r="C156" t="inlineStr">
         <is>
@@ -9354,10 +9046,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B157" t="n">
+        <v>2</v>
       </c>
       <c r="C157" t="inlineStr">
         <is>
@@ -9401,10 +9091,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B158" t="n">
+        <v>2</v>
       </c>
       <c r="C158" t="inlineStr">
         <is>
@@ -9448,10 +9136,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B159" t="n">
+        <v>2</v>
       </c>
       <c r="C159" t="inlineStr">
         <is>
@@ -9495,10 +9181,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B160" t="n">
+        <v>2</v>
       </c>
       <c r="C160" t="inlineStr">
         <is>
@@ -9542,10 +9226,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B161" t="n">
+        <v>2</v>
       </c>
       <c r="C161" t="inlineStr">
         <is>
@@ -9589,10 +9271,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B162" t="n">
+        <v>2</v>
       </c>
       <c r="C162" t="inlineStr">
         <is>
@@ -9636,10 +9316,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B163" t="n">
+        <v>2</v>
       </c>
       <c r="C163" t="inlineStr">
         <is>
@@ -9683,10 +9361,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B164" t="n">
+        <v>2</v>
       </c>
       <c r="C164" t="inlineStr">
         <is>
@@ -9730,10 +9406,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B165" t="n">
+        <v>2</v>
       </c>
       <c r="C165" t="inlineStr">
         <is>
@@ -9777,10 +9451,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B166" t="n">
+        <v>2</v>
       </c>
       <c r="C166" t="inlineStr">
         <is>
@@ -9824,10 +9496,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B167" t="n">
+        <v>2</v>
       </c>
       <c r="C167" t="inlineStr">
         <is>
@@ -9871,10 +9541,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B168" t="n">
+        <v>2</v>
       </c>
       <c r="C168" t="inlineStr">
         <is>
@@ -9918,10 +9586,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B169" t="n">
+        <v>2</v>
       </c>
       <c r="C169" t="inlineStr">
         <is>
@@ -9965,10 +9631,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B170" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B170" t="n">
+        <v>2</v>
       </c>
       <c r="C170" t="inlineStr">
         <is>
@@ -10012,10 +9676,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B171" t="n">
+        <v>2</v>
       </c>
       <c r="C171" t="inlineStr">
         <is>
@@ -10059,10 +9721,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B172" t="n">
+        <v>2</v>
       </c>
       <c r="C172" t="inlineStr">
         <is>
@@ -10106,10 +9766,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B173" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B173" t="n">
+        <v>2</v>
       </c>
       <c r="C173" t="inlineStr">
         <is>
@@ -10153,10 +9811,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B174" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B174" t="n">
+        <v>2</v>
       </c>
       <c r="C174" t="inlineStr">
         <is>
@@ -10200,10 +9856,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B175" t="n">
+        <v>2</v>
       </c>
       <c r="C175" t="inlineStr">
         <is>
@@ -10247,10 +9901,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B176" t="n">
+        <v>2</v>
       </c>
       <c r="C176" t="inlineStr">
         <is>
@@ -10294,10 +9946,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B177" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B177" t="n">
+        <v>2</v>
       </c>
       <c r="C177" t="inlineStr">
         <is>
@@ -10341,10 +9991,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B178" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B178" t="n">
+        <v>2</v>
       </c>
       <c r="C178" t="inlineStr">
         <is>
@@ -10388,10 +10036,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B179" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B179" t="n">
+        <v>2</v>
       </c>
       <c r="C179" t="inlineStr">
         <is>
@@ -10435,10 +10081,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B180" t="n">
+        <v>2</v>
       </c>
       <c r="C180" t="inlineStr">
         <is>
@@ -10482,10 +10126,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B181" t="n">
+        <v>2</v>
       </c>
       <c r="C181" t="inlineStr">
         <is>
@@ -10529,10 +10171,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
+      <c r="B182" t="n">
+        <v>2</v>
       </c>
       <c r="C182" t="inlineStr">
         <is>
@@ -10576,10 +10216,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B183" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B183" t="n">
+        <v>3</v>
       </c>
       <c r="C183" t="inlineStr">
         <is>
@@ -10699,10 +10337,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B184" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B184" t="n">
+        <v>3</v>
       </c>
       <c r="C184" t="inlineStr">
         <is>
@@ -10822,10 +10458,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B185" t="n">
+        <v>3</v>
       </c>
       <c r="C185" t="inlineStr">
         <is>
@@ -10945,10 +10579,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B186" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B186" t="n">
+        <v>3</v>
       </c>
       <c r="C186" t="inlineStr">
         <is>
@@ -11068,10 +10700,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B187" t="n">
+        <v>3</v>
       </c>
       <c r="C187" t="inlineStr">
         <is>
@@ -11191,10 +10821,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B188" t="n">
+        <v>3</v>
       </c>
       <c r="C188" t="inlineStr">
         <is>
@@ -11314,10 +10942,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B189" t="n">
+        <v>3</v>
       </c>
       <c r="C189" t="inlineStr">
         <is>
@@ -11437,10 +11063,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B190" t="n">
+        <v>3</v>
       </c>
       <c r="C190" t="inlineStr">
         <is>
@@ -11560,10 +11184,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B191" t="n">
+        <v>3</v>
       </c>
       <c r="C191" t="inlineStr">
         <is>
@@ -11683,10 +11305,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B192" t="n">
+        <v>3</v>
       </c>
       <c r="C192" t="inlineStr">
         <is>
@@ -11806,10 +11426,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B193" t="n">
+        <v>3</v>
       </c>
       <c r="C193" t="inlineStr">
         <is>
@@ -11853,10 +11471,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B194" t="n">
+        <v>3</v>
       </c>
       <c r="C194" t="inlineStr">
         <is>
@@ -11900,10 +11516,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B195" t="n">
+        <v>3</v>
       </c>
       <c r="C195" t="inlineStr">
         <is>
@@ -11947,10 +11561,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B196" t="n">
+        <v>3</v>
       </c>
       <c r="C196" t="inlineStr">
         <is>
@@ -11994,10 +11606,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B197" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B197" t="n">
+        <v>3</v>
       </c>
       <c r="C197" t="inlineStr">
         <is>
@@ -12041,10 +11651,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B198" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B198" t="n">
+        <v>3</v>
       </c>
       <c r="C198" t="inlineStr">
         <is>
@@ -12088,10 +11696,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B199" t="n">
+        <v>3</v>
       </c>
       <c r="C199" t="inlineStr">
         <is>
@@ -12135,10 +11741,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B200" t="n">
+        <v>3</v>
       </c>
       <c r="C200" t="inlineStr">
         <is>
@@ -12182,10 +11786,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B201" t="n">
+        <v>3</v>
       </c>
       <c r="C201" t="inlineStr">
         <is>
@@ -12229,10 +11831,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B202" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B202" t="n">
+        <v>3</v>
       </c>
       <c r="C202" t="inlineStr">
         <is>
@@ -12276,10 +11876,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B203" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B203" t="n">
+        <v>3</v>
       </c>
       <c r="C203" t="inlineStr">
         <is>
@@ -12323,10 +11921,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B204" t="n">
+        <v>3</v>
       </c>
       <c r="C204" t="inlineStr">
         <is>
@@ -12370,10 +11966,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B205" t="n">
+        <v>3</v>
       </c>
       <c r="C205" t="inlineStr">
         <is>
@@ -12417,10 +12011,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B206" t="n">
+        <v>3</v>
       </c>
       <c r="C206" t="inlineStr">
         <is>
@@ -12464,10 +12056,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B207" t="n">
+        <v>3</v>
       </c>
       <c r="C207" t="inlineStr">
         <is>
@@ -12511,10 +12101,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B208" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B208" t="n">
+        <v>3</v>
       </c>
       <c r="C208" t="inlineStr">
         <is>
@@ -12558,10 +12146,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B209" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B209" t="n">
+        <v>3</v>
       </c>
       <c r="C209" t="inlineStr">
         <is>
@@ -12605,10 +12191,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B210" t="n">
+        <v>3</v>
       </c>
       <c r="C210" t="inlineStr">
         <is>
@@ -12652,10 +12236,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B211" t="n">
+        <v>3</v>
       </c>
       <c r="C211" t="inlineStr">
         <is>
@@ -12699,10 +12281,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B212" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B212" t="n">
+        <v>3</v>
       </c>
       <c r="C212" t="inlineStr">
         <is>
@@ -12746,10 +12326,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B213" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B213" t="n">
+        <v>3</v>
       </c>
       <c r="C213" t="inlineStr">
         <is>
@@ -12793,10 +12371,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B214" t="n">
+        <v>3</v>
       </c>
       <c r="C214" t="inlineStr">
         <is>
@@ -12840,10 +12416,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B215" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B215" t="n">
+        <v>3</v>
       </c>
       <c r="C215" t="inlineStr">
         <is>
@@ -12887,10 +12461,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B216" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B216" t="n">
+        <v>3</v>
       </c>
       <c r="C216" t="inlineStr">
         <is>
@@ -12934,10 +12506,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B217" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B217" t="n">
+        <v>3</v>
       </c>
       <c r="C217" t="inlineStr">
         <is>
@@ -12981,10 +12551,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B218" t="n">
+        <v>3</v>
       </c>
       <c r="C218" t="inlineStr">
         <is>
@@ -13028,10 +12596,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B219" t="n">
+        <v>3</v>
       </c>
       <c r="C219" t="inlineStr">
         <is>
@@ -13075,10 +12641,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B220" t="n">
+        <v>3</v>
       </c>
       <c r="C220" t="inlineStr">
         <is>
@@ -13122,10 +12686,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B221" t="n">
+        <v>3</v>
       </c>
       <c r="C221" t="inlineStr">
         <is>
@@ -13169,10 +12731,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B222" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B222" t="n">
+        <v>3</v>
       </c>
       <c r="C222" t="inlineStr">
         <is>
@@ -13216,10 +12776,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B223" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B223" t="n">
+        <v>3</v>
       </c>
       <c r="C223" t="inlineStr">
         <is>
@@ -13263,10 +12821,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B224" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B224" t="n">
+        <v>3</v>
       </c>
       <c r="C224" t="inlineStr">
         <is>
@@ -13310,10 +12866,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B225" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B225" t="n">
+        <v>3</v>
       </c>
       <c r="C225" t="inlineStr">
         <is>
@@ -13357,10 +12911,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B226" t="n">
+        <v>3</v>
       </c>
       <c r="C226" t="inlineStr">
         <is>
@@ -13404,10 +12956,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B227" t="n">
+        <v>3</v>
       </c>
       <c r="C227" t="inlineStr">
         <is>
@@ -13451,10 +13001,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B228" t="n">
+        <v>3</v>
       </c>
       <c r="C228" t="inlineStr">
         <is>
@@ -13498,10 +13046,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B229" t="n">
+        <v>3</v>
       </c>
       <c r="C229" t="inlineStr">
         <is>
@@ -13545,10 +13091,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B230" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B230" t="n">
+        <v>3</v>
       </c>
       <c r="C230" t="inlineStr">
         <is>
@@ -13592,10 +13136,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B231" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B231" t="n">
+        <v>3</v>
       </c>
       <c r="C231" t="inlineStr">
         <is>
@@ -13639,10 +13181,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+      <c r="B232" t="n">
+        <v>3</v>
       </c>
       <c r="C232" t="inlineStr">
         <is>
@@ -13686,10 +13226,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B233" t="n">
+        <v>4</v>
       </c>
       <c r="C233" t="inlineStr">
         <is>
@@ -13809,10 +13347,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B234" t="n">
+        <v>4</v>
       </c>
       <c r="C234" t="inlineStr">
         <is>
@@ -13932,10 +13468,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B235" t="n">
+        <v>4</v>
       </c>
       <c r="C235" t="inlineStr">
         <is>
@@ -14055,10 +13589,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B236" t="n">
+        <v>4</v>
       </c>
       <c r="C236" t="inlineStr">
         <is>
@@ -14178,10 +13710,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B237" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B237" t="n">
+        <v>4</v>
       </c>
       <c r="C237" t="inlineStr">
         <is>
@@ -14301,10 +13831,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B238" t="n">
+        <v>4</v>
       </c>
       <c r="C238" t="inlineStr">
         <is>
@@ -14424,10 +13952,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B239" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B239" t="n">
+        <v>4</v>
       </c>
       <c r="C239" t="inlineStr">
         <is>
@@ -14547,10 +14073,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B240" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B240" t="n">
+        <v>4</v>
       </c>
       <c r="C240" t="inlineStr">
         <is>
@@ -14670,10 +14194,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B241" t="n">
+        <v>4</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
@@ -14793,10 +14315,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B242" t="n">
+        <v>4</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
@@ -14916,10 +14436,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B243" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B243" t="n">
+        <v>4</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
@@ -14963,10 +14481,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B244" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B244" t="n">
+        <v>4</v>
       </c>
       <c r="C244" t="inlineStr">
         <is>
@@ -15010,10 +14526,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B245" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B245" t="n">
+        <v>4</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
@@ -15057,10 +14571,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B246" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B246" t="n">
+        <v>4</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
@@ -15104,10 +14616,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B247" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B247" t="n">
+        <v>4</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
@@ -15151,10 +14661,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B248" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B248" t="n">
+        <v>4</v>
       </c>
       <c r="C248" t="inlineStr">
         <is>
@@ -15198,10 +14706,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B249" t="n">
+        <v>4</v>
       </c>
       <c r="C249" t="inlineStr">
         <is>
@@ -15245,10 +14751,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B250" t="n">
+        <v>4</v>
       </c>
       <c r="C250" t="inlineStr">
         <is>
@@ -15292,10 +14796,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B251" t="n">
+        <v>4</v>
       </c>
       <c r="C251" t="inlineStr">
         <is>
@@ -15339,10 +14841,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B252" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B252" t="n">
+        <v>4</v>
       </c>
       <c r="C252" t="inlineStr">
         <is>
@@ -15386,10 +14886,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B253" t="n">
+        <v>4</v>
       </c>
       <c r="C253" t="inlineStr">
         <is>
@@ -15433,10 +14931,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B254" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B254" t="n">
+        <v>4</v>
       </c>
       <c r="C254" t="inlineStr">
         <is>
@@ -15480,10 +14976,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B255" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B255" t="n">
+        <v>4</v>
       </c>
       <c r="C255" t="inlineStr">
         <is>
@@ -15527,10 +15021,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B256" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B256" t="n">
+        <v>4</v>
       </c>
       <c r="C256" t="inlineStr">
         <is>
@@ -15574,10 +15066,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B257" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B257" t="n">
+        <v>4</v>
       </c>
       <c r="C257" t="inlineStr">
         <is>
@@ -15621,10 +15111,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B258" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B258" t="n">
+        <v>4</v>
       </c>
       <c r="C258" t="inlineStr">
         <is>
@@ -15668,10 +15156,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B259" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B259" t="n">
+        <v>4</v>
       </c>
       <c r="C259" t="inlineStr">
         <is>
@@ -15715,10 +15201,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B260" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B260" t="n">
+        <v>4</v>
       </c>
       <c r="C260" t="inlineStr">
         <is>
@@ -15762,10 +15246,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B261" t="n">
+        <v>4</v>
       </c>
       <c r="C261" t="inlineStr">
         <is>
@@ -15809,10 +15291,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B262" t="n">
+        <v>4</v>
       </c>
       <c r="C262" t="inlineStr">
         <is>
@@ -15856,10 +15336,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B263" t="n">
+        <v>4</v>
       </c>
       <c r="C263" t="inlineStr">
         <is>
@@ -15903,10 +15381,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B264" t="n">
+        <v>4</v>
       </c>
       <c r="C264" t="inlineStr">
         <is>
@@ -15950,10 +15426,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B265" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B265" t="n">
+        <v>4</v>
       </c>
       <c r="C265" t="inlineStr">
         <is>
@@ -15997,10 +15471,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B266" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B266" t="n">
+        <v>4</v>
       </c>
       <c r="C266" t="inlineStr">
         <is>
@@ -16044,10 +15516,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B267" t="n">
+        <v>4</v>
       </c>
       <c r="C267" t="inlineStr">
         <is>
@@ -16091,10 +15561,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B268" t="n">
+        <v>4</v>
       </c>
       <c r="C268" t="inlineStr">
         <is>
@@ -16138,10 +15606,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B269" t="n">
+        <v>4</v>
       </c>
       <c r="C269" t="inlineStr">
         <is>
@@ -16185,10 +15651,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B270" t="n">
+        <v>4</v>
       </c>
       <c r="C270" t="inlineStr">
         <is>
@@ -16232,10 +15696,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B271" t="n">
+        <v>4</v>
       </c>
       <c r="C271" t="inlineStr">
         <is>
@@ -16279,10 +15741,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B272" t="n">
+        <v>4</v>
       </c>
       <c r="C272" t="inlineStr">
         <is>
@@ -16326,10 +15786,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B273" t="n">
+        <v>4</v>
       </c>
       <c r="C273" t="inlineStr">
         <is>
@@ -16373,10 +15831,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B274" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B274" t="n">
+        <v>4</v>
       </c>
       <c r="C274" t="inlineStr">
         <is>
@@ -16420,10 +15876,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B275" t="n">
+        <v>4</v>
       </c>
       <c r="C275" t="inlineStr">
         <is>
@@ -16467,10 +15921,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B276" t="n">
+        <v>4</v>
       </c>
       <c r="C276" t="inlineStr">
         <is>
@@ -16514,10 +15966,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B277" t="n">
+        <v>4</v>
       </c>
       <c r="C277" t="inlineStr">
         <is>
@@ -16561,10 +16011,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B278" t="n">
+        <v>4</v>
       </c>
       <c r="C278" t="inlineStr">
         <is>
@@ -16608,10 +16056,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B279" t="n">
+        <v>4</v>
       </c>
       <c r="C279" t="inlineStr">
         <is>
@@ -16655,10 +16101,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B280" t="n">
+        <v>4</v>
       </c>
       <c r="C280" t="inlineStr">
         <is>
@@ -16702,10 +16146,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B281" t="n">
+        <v>4</v>
       </c>
       <c r="C281" t="inlineStr">
         <is>
@@ -16749,10 +16191,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+      <c r="B282" t="n">
+        <v>4</v>
       </c>
       <c r="C282" t="inlineStr">
         <is>
@@ -16796,10 +16236,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B283" t="n">
+        <v>5</v>
       </c>
       <c r="C283" t="inlineStr">
         <is>
@@ -16919,10 +16357,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B284" t="n">
+        <v>5</v>
       </c>
       <c r="C284" t="inlineStr">
         <is>
@@ -17042,10 +16478,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B285" t="n">
+        <v>5</v>
       </c>
       <c r="C285" t="inlineStr">
         <is>
@@ -17165,10 +16599,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B286" t="n">
+        <v>5</v>
       </c>
       <c r="C286" t="inlineStr">
         <is>
@@ -17288,10 +16720,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B287" t="n">
+        <v>5</v>
       </c>
       <c r="C287" t="inlineStr">
         <is>
@@ -17411,10 +16841,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B288" t="n">
+        <v>5</v>
       </c>
       <c r="C288" t="inlineStr">
         <is>
@@ -17534,10 +16962,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B289" t="n">
+        <v>5</v>
       </c>
       <c r="C289" t="inlineStr">
         <is>
@@ -17657,10 +17083,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B290" t="n">
+        <v>5</v>
       </c>
       <c r="C290" t="inlineStr">
         <is>
@@ -17780,10 +17204,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B291" t="n">
+        <v>5</v>
       </c>
       <c r="C291" t="inlineStr">
         <is>
@@ -17903,10 +17325,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B292" t="n">
+        <v>5</v>
       </c>
       <c r="C292" t="inlineStr">
         <is>
@@ -18026,10 +17446,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B293" t="n">
+        <v>5</v>
       </c>
       <c r="C293" t="inlineStr">
         <is>
@@ -18073,10 +17491,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B294" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B294" t="n">
+        <v>5</v>
       </c>
       <c r="C294" t="inlineStr">
         <is>
@@ -18120,10 +17536,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B295" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B295" t="n">
+        <v>5</v>
       </c>
       <c r="C295" t="inlineStr">
         <is>
@@ -18167,10 +17581,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B296" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B296" t="n">
+        <v>5</v>
       </c>
       <c r="C296" t="inlineStr">
         <is>
@@ -18214,10 +17626,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B297" t="n">
+        <v>5</v>
       </c>
       <c r="C297" t="inlineStr">
         <is>
@@ -18261,10 +17671,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B298" t="n">
+        <v>5</v>
       </c>
       <c r="C298" t="inlineStr">
         <is>
@@ -18308,10 +17716,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B299" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B299" t="n">
+        <v>5</v>
       </c>
       <c r="C299" t="inlineStr">
         <is>
@@ -18355,10 +17761,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B300" t="n">
+        <v>5</v>
       </c>
       <c r="C300" t="inlineStr">
         <is>
@@ -18402,10 +17806,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B301" t="n">
+        <v>5</v>
       </c>
       <c r="C301" t="inlineStr">
         <is>
@@ -18449,10 +17851,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B302" t="n">
+        <v>5</v>
       </c>
       <c r="C302" t="inlineStr">
         <is>
@@ -18496,10 +17896,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B303" t="n">
+        <v>5</v>
       </c>
       <c r="C303" t="inlineStr">
         <is>
@@ -18543,10 +17941,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B304" t="n">
+        <v>5</v>
       </c>
       <c r="C304" t="inlineStr">
         <is>
@@ -18590,10 +17986,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B305" t="n">
+        <v>5</v>
       </c>
       <c r="C305" t="inlineStr">
         <is>
@@ -18637,10 +18031,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B306" t="n">
+        <v>5</v>
       </c>
       <c r="C306" t="inlineStr">
         <is>
@@ -18684,10 +18076,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B307" t="n">
+        <v>5</v>
       </c>
       <c r="C307" t="inlineStr">
         <is>
@@ -18731,10 +18121,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B308" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B308" t="n">
+        <v>5</v>
       </c>
       <c r="C308" t="inlineStr">
         <is>
@@ -18778,10 +18166,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B309" t="n">
+        <v>5</v>
       </c>
       <c r="C309" t="inlineStr">
         <is>
@@ -18825,10 +18211,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B310" t="n">
+        <v>5</v>
       </c>
       <c r="C310" t="inlineStr">
         <is>
@@ -18872,10 +18256,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B311" t="n">
+        <v>5</v>
       </c>
       <c r="C311" t="inlineStr">
         <is>
@@ -18919,10 +18301,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B312" t="n">
+        <v>5</v>
       </c>
       <c r="C312" t="inlineStr">
         <is>
@@ -18966,10 +18346,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B313" t="n">
+        <v>5</v>
       </c>
       <c r="C313" t="inlineStr">
         <is>
@@ -19013,10 +18391,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B314" t="n">
+        <v>5</v>
       </c>
       <c r="C314" t="inlineStr">
         <is>
@@ -19060,10 +18436,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B315" t="n">
+        <v>5</v>
       </c>
       <c r="C315" t="inlineStr">
         <is>
@@ -19107,10 +18481,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B316" t="n">
+        <v>5</v>
       </c>
       <c r="C316" t="inlineStr">
         <is>
@@ -19154,10 +18526,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B317" t="n">
+        <v>5</v>
       </c>
       <c r="C317" t="inlineStr">
         <is>
@@ -19201,10 +18571,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B318" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B318" t="n">
+        <v>5</v>
       </c>
       <c r="C318" t="inlineStr">
         <is>
@@ -19248,10 +18616,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B319" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B319" t="n">
+        <v>5</v>
       </c>
       <c r="C319" t="inlineStr">
         <is>
@@ -19295,10 +18661,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B320" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B320" t="n">
+        <v>5</v>
       </c>
       <c r="C320" t="inlineStr">
         <is>
@@ -19342,10 +18706,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B321" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B321" t="n">
+        <v>5</v>
       </c>
       <c r="C321" t="inlineStr">
         <is>
@@ -19389,10 +18751,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B322" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B322" t="n">
+        <v>5</v>
       </c>
       <c r="C322" t="inlineStr">
         <is>
@@ -19436,10 +18796,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B323" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B323" t="n">
+        <v>5</v>
       </c>
       <c r="C323" t="inlineStr">
         <is>
@@ -19483,10 +18841,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B324" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B324" t="n">
+        <v>5</v>
       </c>
       <c r="C324" t="inlineStr">
         <is>
@@ -19530,10 +18886,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B325" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B325" t="n">
+        <v>5</v>
       </c>
       <c r="C325" t="inlineStr">
         <is>
@@ -19577,10 +18931,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B326" t="n">
+        <v>5</v>
       </c>
       <c r="C326" t="inlineStr">
         <is>
@@ -19624,10 +18976,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B327" t="n">
+        <v>5</v>
       </c>
       <c r="C327" t="inlineStr">
         <is>
@@ -19671,10 +19021,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B328" t="n">
+        <v>5</v>
       </c>
       <c r="C328" t="inlineStr">
         <is>
@@ -19718,10 +19066,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B329" t="n">
+        <v>5</v>
       </c>
       <c r="C329" t="inlineStr">
         <is>
@@ -19765,10 +19111,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B330" t="n">
+        <v>5</v>
       </c>
       <c r="C330" t="inlineStr">
         <is>
@@ -19812,10 +19156,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B331" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B331" t="n">
+        <v>5</v>
       </c>
       <c r="C331" t="inlineStr">
         <is>
@@ -19859,10 +19201,8 @@
           <t>Текстово-графическое</t>
         </is>
       </c>
-      <c r="B332" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
+      <c r="B332" t="n">
+        <v>5</v>
       </c>
       <c r="C332" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fix all Direct errors: minus slash, text length, title length
</commit_message>
<xml_diff>
--- a/direct_voronezh_krovstroyrf.xlsx
+++ b/direct_voronezh_krovstroyrf.xlsx
@@ -618,7 +618,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z3" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -868,7 +868,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z10" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1203,7 +1203,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1218,7 +1218,7 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z17" t="inlineStr">
@@ -1443,7 +1443,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1458,7 +1458,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1553,7 +1553,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1668,7 +1668,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z24" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1918,7 +1918,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z31" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -2368,7 +2368,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z38" t="inlineStr">
@@ -2493,7 +2493,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2508,7 +2508,7 @@
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
@@ -2718,7 +2718,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z45" t="inlineStr">
@@ -2843,7 +2843,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2858,7 +2858,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2968,7 +2968,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z52" t="inlineStr">
@@ -3193,7 +3193,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3208,7 +3208,7 @@
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3318,7 +3318,7 @@
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
@@ -3418,7 +3418,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z59" t="inlineStr">
@@ -3543,7 +3543,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3558,7 +3558,7 @@
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J64" t="inlineStr">
@@ -3653,7 +3653,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -3668,7 +3668,7 @@
       </c>
       <c r="I65" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J65" t="inlineStr">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -б/у -бу -продаю -продам</t>
+          <t>-своими руками -видео -инструкция -бесплатно -схема -чертеж -расчет -материалы -купить -магазин -работа -вакансия -резюме -обучение -курсы -бу -продаю -продам</t>
         </is>
       </c>
       <c r="Z66" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Кровельные работы в Воронеж под ключ</t>
+          <t>Кровля под ключ в Воронеж</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -3908,7 +3908,7 @@
       </c>
       <c r="I71" t="inlineStr">
         <is>
-          <t>Кровля под ключ. Гарантия до 39 лет. Русские бригады. Фиксированная цена без доп. расходов!</t>
+          <t>Гарантия до 39 лет. Русские бригады. Фикс. цена без доп. расходов!</t>
         </is>
       </c>
       <c r="J71" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Ремонт кровли в Воронеж — Гарантия 39 лет!</t>
+          <t>Ремонт кровли Воронеж. Гарантия</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -4018,7 +4018,7 @@
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5% при заказе сегодня!</t>
+          <t>3 бригады. Гарантия 39 лет. Бесплатный выезд на замер. Скидка 5%!</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">

</xml_diff>